<commit_message>
Add limma/limma-full rows to metabolomics v2 example; clean stale outputs
Adds a limma and a limma-full row (HFD-Dam over RD-Dam) to
comparisons-metabolomics-v2.xlsx so example 1 demonstrates both test
types. Verified in a scratch run: both produce full output sets and a
PowerPoint report, with fold changes identical to the t-test and
moderated p-values closely tracking it.

Removes 75 superseded files from examples/results-metabolomics_v2:
outputs written under the fork's old naming (before the test type was
appended to filenames) and three empty run logs. Each output has a
current-named counterpart from the rerun.

Ignores regenerated example outputs (examples/results-*/) going
forward. Already-tracked output files are unaffected.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/comparisons-metabolomics-v2.xlsx
+++ b/examples/comparisons-metabolomics-v2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t xml:space="preserve">SampleID</t>
   </si>
@@ -193,6 +193,12 @@
   </si>
   <si>
     <t xml:space="preserve">MaleMRD,MaleMHFD,FemMRD,FemMHFD,RD-Dam,HFD-Dam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">limma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">limma-full</t>
   </si>
 </sst>
 </file>
@@ -942,6 +948,42 @@
         <v>59</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1</v>
+      </c>
+      <c r="F6"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>1</v>
+      </c>
+      <c r="F7"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>